<commit_message>
Refresh Excel for date filters and Reckitt mapping fixes.
Document Order ENTRY_TIME and Customer DATECREATED filters, Invoice toDate 23:59:59, and Karl field updates. Keep the four existing sheets.

Co-authored-by: soniarun532-rgb <soniarun532-rgb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/postman/SAT-Datashare-SAPI-PAPI-EAPI-payloads (3) (2).xlsx
+++ b/postman/SAT-Datashare-SAPI-PAPI-EAPI-payloads (3) (2).xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,6 +46,9 @@
       <name val="Calibri"/>
       <b val="1"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -98,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -119,6 +122,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -692,10 +698,7 @@
       <c r="D2" s="2" t="inlineStr">
         <is>
           <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
+            <rPr/>
             <t xml:space="preserve">SHOPID -&gt; STOREID
 DISCOUNT -&gt; Discount
 USERID -&gt; SalesRepID
@@ -705,18 +708,23 @@
           </r>
           <r>
             <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>papi.sat.solutech.distributor.id (1000097205)</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> -&gt; DistributorID
+              <b val="1"/>
+            </rPr>
+            <t>papi.sat.solutech.distributor.id</t>
+          </r>
+          <r>
+            <rPr/>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>1000097205</t>
+          </r>
+          <r>
+            <rPr/>
+            <t xml:space="preserve">) -&gt; DistributorID
 PRODUCT_CODE -&gt; ProductID  (strip leading letters)
 SUPPLIER_ID -&gt; WarehouseID
 SALE_ORDER_ID -&gt; OrderNumber
@@ -729,20 +737,25 @@
           </r>
           <r>
             <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>papi.sat.solutech.currency (KES)</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> -&gt; Currency
+              <b val="1"/>
+            </rPr>
+            <t>papi.sat.solutech.currency</t>
+          </r>
+          <r>
+            <rPr/>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>KES</t>
+          </r>
+          <r>
+            <rPr/>
+            <t>) -&gt; Currency
 QUANTITY -&gt; QuantityInvoiced
-VALUE_SOLD -&gt; AmountInvoiced
+VALUE_SOLD -&gt; AmountInvoiced  (PAPI amount2, 2 decimals, format 0.00)
 ENTRY_TYPE -&gt; TransType</t>
           </r>
         </is>
@@ -753,7 +766,7 @@
 from {database}.bi_salesmaster as a
 left join {database}.bi_customer_visits as b on a.VisitID = b.visitid
 inner join {database}.bi_products as c on a.PRODUCT_ID = c.id and c.supplier = '{supplier}'
-where a.Created_AT between '&lt;fromDate&gt; 00:00:00' and '&lt;toDate&gt; 00:00:00'
+where a.Created_AT between '&lt;fromDate&gt; 00:00:00' and '&lt;toDate&gt; 23:59:59'
 order by a.Entry_ID desc
 LIMIT &lt;pageSize + 1&gt; OFFSET &lt;pageNumber * pageSize&gt;</t>
         </is>
@@ -792,7 +805,7 @@
           </r>
           <r>
             <rPr/>
-            <t>, VAT 2 decimals, ProductID numeric, InvoiceStatus from DELIVERED</t>
+            <t>, VAT and AmountInvoiced 2 decimals, ProductID numeric, InvoiceStatus from DELIVERED, toDate 23:59:59</t>
           </r>
         </is>
       </c>
@@ -871,19 +884,26 @@
       <c r="C3" s="3" t="inlineStr">
         <is>
           <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
+            <rPr/>
             <t xml:space="preserve"> {
             "StoreID": 1801,
             "SalesRepID": 89,
             "RouteID": "",
             "ProductID": "969584",
-            "DistributorID": "???",
+            "DistributorID": </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>"1000097205"</t>
+          </r>
+          <r>
+            <rPr/>
+            <t xml:space="preserve">,
             "WarehouseID": 183,
             "OrderNumber": 69,
-            "OrderDate": "",
+            "OrderDate": "10/09/2026",
             "OrderStartTime": "",
             "OrderEndTime": "",
             "OrderStatus": "Cancelled",
@@ -892,20 +912,15 @@
           </r>
           <r>
             <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
+              <b val="1"/>
             </rPr>
             <t>"KES"</t>
           </r>
           <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
+            <rPr/>
             <t>,
             "QuantityOrdered": 1,
-            "AmountOrdered": 372,
+            "AmountOrdered": "372.00",
             "Discount": 0,
             "VATAmount": "51.31"
         }</t>
@@ -915,18 +930,35 @@
       <c r="D3" s="3" t="inlineStr">
         <is>
           <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
+            <rPr/>
             <t xml:space="preserve">SHOP_ID -&gt; StoreID
 USER_ID -&gt; SalesRepID  (not SALES_REP name)
 ROUTEID -&gt; RouteID
 PRODUCT_CODE -&gt; ProductID  (strip leading letters)
-hardcoded '???' -&gt; DistributorID
+</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>papi.sat.solutech.distributor.id</t>
+          </r>
+          <r>
+            <rPr/>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>1000097205</t>
+          </r>
+          <r>
+            <rPr/>
+            <t xml:space="preserve">) -&gt; DistributorID
 SUPPLIER_ID -&gt; WarehouseID
 ENTRY_ID -&gt; OrderNumber
-CHECKINTIME -&gt; OrderDate  (dd/MM/yyyy)
+ENTRY_TIME -&gt; OrderDate  (dd/MM/yyyy)
 CHECKINTIME -&gt; OrderStartTime  (HH:mm:ss)
 CHECKOUTTIME -&gt; OrderEndTime  (HH:mm:ss)
 DELIVERED -&gt; OrderStatus
@@ -935,20 +967,25 @@
           </r>
           <r>
             <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <sz val="10"/>
-            </rPr>
-            <t>papi.sat.solutech.currency (KES)</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve"> -&gt; Currency
+              <b val="1"/>
+            </rPr>
+            <t>papi.sat.solutech.currency</t>
+          </r>
+          <r>
+            <rPr/>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>KES</t>
+          </r>
+          <r>
+            <rPr/>
+            <t>) -&gt; Currency
 QUANTITY -&gt; QuantityOrdered
-TOTAL_VAT_INC -&gt; AmountOrdered
+TOTAL_VAT_INC -&gt; AmountOrdered  (PAPI amount2, 2 decimals)
 DISCOUNT -&gt; Discount
 TOTAL_VAT -&gt; VATAmount  (PAPI amount2, 2 decimals)</t>
           </r>
@@ -960,9 +997,9 @@
 from {database}.bi_ordersmaster as a
 inner join {database}.bi_products as c on a.PRODUCT_ID = c.id and c.supplier = '{supplier}'
 left join {database}.bi_customer_visits as b on a.VISIT_ID = b.visitid
+where a.ENTRY_TIME between '&lt;fromDate&gt; 00:00:00' and '&lt;toDate&gt; 23:59:59'
 order by a.ENTRY_ID desc
-LIMIT &lt;pageSize + 1&gt; OFFSET &lt;pageNumber * pageSize&gt;
-Note: Exp/PAPI still send fromDate and toDate. Current SAPI Order SQL does not filter on those dates.</t>
+LIMIT &lt;pageSize + 1&gt; OFFSET &lt;pageNumber * pageSize&gt;</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -987,7 +1024,20 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>UPDATED — SalesRepID = USER_ID, ProductID numeric, VAT 2 decimals</t>
+          <r>
+            <rPr/>
+            <t xml:space="preserve">UPDATED — SalesRepID = USER_ID, OrderDate from ENTRY_TIME, DistributorID </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>1000097205</t>
+          </r>
+          <r>
+            <rPr/>
+            <t>, AmountOrdered 2 decimals, date filter on ENTRY_TIME</t>
+          </r>
         </is>
       </c>
     </row>
@@ -1403,7 +1453,7 @@
             "StoreCategory": "RETAIL SHOP",
             "Channel": "GENERAL TRADE",
             "StoreClassification": "GENERAL TRADE",
-            "WarehouseID": "???",
+            "WarehouseID": null,
             "Longitude": 36.9328219,
             "Latitude": -1.2349905,
             "City": "RUIRU",
@@ -1422,7 +1472,7 @@
 CUSTOMERCATEGORY -&gt; StoreCategory
 CHANNEL -&gt; Channel
 CHANNEL -&gt; StoreClassification
-hardcoded '???' -&gt; WarehouseID
+null -&gt; WarehouseID
 LONGITUDE -&gt; Longitude
 LATITUDE -&gt; Latitude
 LOCATIONNAME -&gt; City
@@ -1438,6 +1488,7 @@
           <t>Select a.*
 from {database}.bi_customer_master as a
 where a.Customer_Type = 'Customer'
+and a.DATECREATED between '&lt;fromDate&gt; 00:00:00' and '&lt;toDate&gt; 23:59:59'
 and exists (
   Select 1 from (
     Select distinct SHOPID from (
@@ -1451,8 +1502,7 @@
   where w.SHOPID = a.SHOPID
 )
 order by a.SHOPID
-LIMIT &lt;pageSize + 1&gt; OFFSET &lt;pageNumber * pageSize&gt;
-Note: Exp/PAPI send fromDate and toDate. Current SAPI Customer SQL does not filter on those dates.</t>
+LIMIT &lt;pageSize + 1&gt; OFFSET &lt;pageNumber * pageSize&gt;</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -1477,7 +1527,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>Unchanged mapping</t>
+          <t>UPDATED — WarehouseID null, DATECREATED date filter</t>
         </is>
       </c>
     </row>
@@ -1507,7 +1557,7 @@
             "DistributorWarehouseCode": "",
             "Date": "17/08/2026",
             "InventoryQuantity": -880,
-            "InventoryPrice": 1060
+            "InventoryPrice": null
         }</t>
         </is>
       </c>
@@ -1518,7 +1568,7 @@
 stockpoint_name -&gt; DistributorWarehouseCode
 date_created -&gt; Date  (dd/MM/yyyy)
 quantity -&gt; InventoryQuantity  (goodsin minus goodsout)
-total_cost -&gt; InventoryPrice</t>
+null -&gt; InventoryPrice</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1560,7 +1610,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>UPDATED — quantity = goodsin minus goodsout</t>
+          <t>UPDATED — quantity = goodsin minus goodsout, InventoryPrice null</t>
         </is>
       </c>
     </row>
@@ -1623,18 +1673,54 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> {
+          <r>
+            <rPr/>
+            <t xml:space="preserve"> {
             "WarehouseID": 183,
             "WarehouseName": "GIKAMBURA STOCKPOINT",
-            "DistributorID": ""
+            "DistributorID": </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>"1000097205"</t>
+          </r>
+          <r>
+            <rPr/>
+            <t xml:space="preserve">
         }</t>
+          </r>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>ID -&gt; WarehouseID
+          <r>
+            <rPr/>
+            <t xml:space="preserve">ID -&gt; WarehouseID
 CUSTOMERNAME -&gt; WarehouseName
-'' -&gt; DistributorID</t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>papi.sat.solutech.distributor.id</t>
+          </r>
+          <r>
+            <rPr/>
+            <t xml:space="preserve"> (</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>1000097205</t>
+          </r>
+          <r>
+            <rPr/>
+            <t>) -&gt; DistributorID</t>
+          </r>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -1672,7 +1758,20 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>Unchanged mapping. EXISTS still commented.</t>
+          <r>
+            <rPr/>
+            <t xml:space="preserve">UPDATED — DistributorID </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>1000097205</t>
+          </r>
+          <r>
+            <rPr/>
+            <t>. EXISTS still commented.</t>
+          </r>
         </is>
       </c>
     </row>
@@ -2160,7 +2259,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>amount2 format 0.00</t>
         </is>
       </c>
     </row>
@@ -2285,14 +2384,38 @@
           <t>DistributorID</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>hardcoded</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>'???' still in PAPI DWL</t>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>papi.sat.solutech.distributor.id</t>
+          </r>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr/>
+            <t xml:space="preserve">property </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>papi.sat.solutech.distributor.id</t>
+          </r>
+          <r>
+            <rPr/>
+            <t xml:space="preserve"> = </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>1000097205</t>
+          </r>
         </is>
       </c>
     </row>
@@ -2353,7 +2476,7 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>CHECKINTIME</t>
+          <t>ENTRY_TIME</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -2548,7 +2671,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>amount2 format 0.00</t>
         </is>
       </c>
     </row>
@@ -3061,14 +3184,10 @@
           <t>WarehouseID</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>hardcoded</t>
-        </is>
-      </c>
+      <c r="C56" s="2" t="n"/>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>'???' still in PAPI DWL</t>
+          <t>null</t>
         </is>
       </c>
     </row>
@@ -3361,14 +3480,10 @@
           <t>InventoryPrice</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>total_cost</t>
-        </is>
-      </c>
+      <c r="C70" s="2" t="n"/>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>null</t>
         </is>
       </c>
     </row>
@@ -3427,10 +3542,38 @@
           <t>DistributorID</t>
         </is>
       </c>
-      <c r="C73" s="3" t="n"/>
-      <c r="D73" s="3" t="inlineStr">
-        <is>
-          <t>empty</t>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>papi.sat.solutech.distributor.id</t>
+          </r>
+        </is>
+      </c>
+      <c r="D73" s="8" t="inlineStr">
+        <is>
+          <r>
+            <rPr/>
+            <t xml:space="preserve">property </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>papi.sat.solutech.distributor.id</t>
+          </r>
+          <r>
+            <rPr/>
+            <t xml:space="preserve"> = </t>
+          </r>
+          <r>
+            <rPr>
+              <b val="1"/>
+            </rPr>
+            <t>1000097205</t>
+          </r>
         </is>
       </c>
     </row>

</xml_diff>